<commit_message>
Setup kit web app (steps 1, 2, 4), PubMed/reference/PDF intake, clean-up review, sample check; extraction fixes
- Local FastAPI app: branding, publication bank (PDF folder, reference export, PubMed IDs), clean-up review with topic check,
  and a 'Check a sample' step with price estimate and scorecard
- Parser fix for 'Material and Methods' headings; whole-paper read when key sections are missing
- Template rule updates after the DADA2 hand check; VCP overlay draft

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/core/extraction_core.xlsx
+++ b/core/extraction_core.xlsx
@@ -639,7 +639,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>If a paper does several things, pick the primary one (the one the title and abstract emphasize). Reviews, guidelines and consensus statements summarize other work. Use 'Other/off-topic' when the paper is not about the disease or genes named in the Context rule (for example an unrelated disease, or a paper that only uses a tool or name that happens to match); say so in the rationale.</t>
+          <t>If a paper does several things, pick the primary one (the one the title and abstract emphasize). Reviews, guidelines and consensus statements summarize other work. Use 'Other/off-topic' when the paper is not about the disease or genes named in the Context rule (for example an unrelated disease, or a paper that only uses a tool or name that happens to match); say so in the rationale. Put design details in the 'detail' field (for example retrospective, prospective, multicenter, randomized, long-term follow-up); empty string if not stated.</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Copy catalog numbers exactly as printed (for example 'ab12345' or '#4691'). Leave the catalog number empty when none is printed; never guess one. Reagents matter because antibody differences can explain contradictory results between papers.</t>
+          <t>Copy catalog numbers exactly as printed (for example 'ab12345' or '#4691'). Leave the catalog number empty when none is printed; never guess one. Reagents matter because antibody differences can explain contradictory results between papers. If the status is Not found and the paper mentions supplementary material, a supplementary table or reagent list that is not in the text, say so in the rationale (the supplement is not part of the library).</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -1133,17 +1133,17 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Author(s) the paper itself labels as corresponding author, usually on the first page or in a footnote.</t>
+          <t>Author(s) the paper itself labels as corresponding author, usually on the first page or in a footnote. An author whose email address is printed as the contact (in a correspondence line, footnote or author block), or who carries an asterisk or envelope symbol that the paper links to correspondence, is a corresponding author.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>The first or last author, unless the paper labels them as corresponding. Email addresses.</t>
+          <t>The first or last author, unless the paper labels them as corresponding or gives them as the contact (by email address or a linked asterisk). Email addresses of people who are not authors.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Look for 'Correspondence to', 'Corresponding author', 'Address correspondence to', 'To whom correspondence should be addressed', or an asterisk/envelope footnote. There can be several: list every one. Give the institution if stated. If the paper labels none, do not guess.</t>
+          <t>Look for 'Correspondence to', 'Corresponding author', 'Address correspondence to', 'To whom correspondence should be addressed', or an asterisk/envelope footnote. There can be several: list every one. Give the institution if stated. An email address printed for an author counts as that author being a corresponding author (Medium confidence when there is no explicit label); in a short paper where every author has an email, list them all. If the paper gives no label, no email and no linked symbol, do not guess.</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -1153,7 +1153,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>The paper labels no corresponding author (common when only email addresses appear in a footnote).</t>
+          <t>The paper gives no correspondence label, no author email address and no linked asterisk or envelope symbol.</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>High when explicitly labelled; Medium when inferred from an email footnote.</t>
+          <t>High when explicitly labelled; Medium when inferred from an email address or a linked asterisk.</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Use the listed treatment class and name the specific drug or regimen in the detail field (for example 'adalimumab').</t>
+          <t>Use the listed treatment class and name the specific drug or regimen in the detail field (for example 'adalimumab'). Make one entry per specific drug or regimen: if a paper uses prednisone and dexamethasone, record two entries (each in its class, each naming its drug in the detail field); never combine several drugs into one entry.</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1332,7 +1332,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1397,52 +1397,52 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>gene_focus</t>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>study_type</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>detail</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>pick-list</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Target gene or protein; Related gene or protein; Both; Other/none</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>The gene or protein the paper is about.</t>
+          <t>Design details such as retrospective, prospective, multicenter, randomized or long-term follow-up; empty string if not stated.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>mutations</t>
+          <t>gene_focus</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>gene</t>
+          <t>value</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr"/>
+          <t>pick-list</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Target gene or protein; Related gene or protein; Both; Other/none</t>
+        </is>
+      </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Gene symbol, for example BRCA1.</t>
+          <t>The gene or protein the paper is about. Support it with a sentence from the paper's own aims, methods or results, not a definition of the gene or disease.</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1454,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>variant</t>
+          <t>gene</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1465,7 +1465,7 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Variant in one-letter protein form (p.R169Q), or the DNA-level change if no protein change is given.</t>
+          <t>Gene symbol, for example BRCA1.</t>
         </is>
       </c>
     </row>
@@ -1477,7 +1477,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>as_written</t>
+          <t>variant</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1488,34 +1488,30 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>The variant exactly as the paper writes it.</t>
+          <t>Variant in one-letter protein form (p.R169Q), or the DNA-level change if no protein change is given.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>model_systems</t>
+          <t>mutations</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>system</t>
+          <t>as_written</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>pick-list</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Human patients; Healthy donors; Primary human cells; Human cell line; Mouse; Zebrafish; Other animal; Yeast/fungus; Recombinant protein; Other</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>The model system.</t>
+          <t>The variant exactly as the paper writes it.</t>
         </is>
       </c>
     </row>
@@ -1527,45 +1523,45 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>system</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
+          <t>pick-list</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Human patients; Healthy donors; Primary human cells; Human cell line; Mouse; Zebrafish; Other animal; Yeast/fungus; Recombinant protein; Other</t>
+        </is>
+      </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Specifics such as cell line name or mouse strain; required if 'Other'; empty string if none.</t>
+          <t>The model system.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>techniques</t>
+          <t>model_systems</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>technique</t>
+          <t>detail</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>pick-list</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Sanger sequencing; Whole-exome sequencing; Gene panel/NGS; Western blot; Flow cytometry; qPCR; ELISA; RNA-seq; Single-cell RNA-seq; Immunohistochemistry; Mass spectrometry; Cytokine/interferon signature; Imaging (MRI/MRA); Biopsy/histology; CRISPR; Crystallography/structure; Other</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>The technique.</t>
+          <t>Specifics such as cell line name or mouse strain; required if 'Other'; empty string if none.</t>
         </is>
       </c>
     </row>
@@ -1577,45 +1573,45 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>technique</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr"/>
+          <t>pick-list</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Sanger sequencing; Whole-exome sequencing; Gene panel/NGS; Western blot; Flow cytometry; qPCR; ELISA; RNA-seq; Single-cell RNA-seq; Immunohistochemistry; Mass spectrometry; Cytokine/interferon signature; Imaging (MRI/MRA); Biopsy/histology; CRISPR; Crystallography/structure; Other</t>
+        </is>
+      </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Required if 'Other' (name the technique); otherwise optional; empty string if none.</t>
+          <t>The technique.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>sample_sources</t>
+          <t>techniques</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>detail</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>pick-list</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Serum; Plasma; PBMC; Whole blood; Bone marrow; Skin biopsy; Fibroblasts; CSF; Urine; Other tissue; Other</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>The sample type.</t>
+          <t>Required if 'Other' (name the technique); otherwise optional; empty string if none.</t>
         </is>
       </c>
     </row>
@@ -1627,30 +1623,34 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>source</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr"/>
+          <t>pick-list</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Serum; Plasma; PBMC; Whole blood; Bone marrow; Skin biopsy; Fibroblasts; CSF; Urine; Other tissue; Other</t>
+        </is>
+      </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Required if 'Other'; otherwise optional (for example patient vs. control); empty string if none.</t>
+          <t>The sample type.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>reagents</t>
+          <t>sample_sources</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>detail</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1661,7 +1661,7 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>The reagent, for example 'anti-[target] antibody' or a specific clone.</t>
+          <t>Required if 'Other'; otherwise optional (for example patient vs. control); empty string if none.</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>vendor</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1684,7 +1684,7 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Supplier if stated; otherwise an empty string.</t>
+          <t>The reagent, for example 'anti-[target] antibody' or a specific clone.</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>catalog_number</t>
+          <t>vendor</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1707,7 +1707,7 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Catalog number EXACTLY as printed; empty string if not reported. Never guess.</t>
+          <t>Supplier if stated; otherwise an empty string.</t>
         </is>
       </c>
     </row>
@@ -1719,7 +1719,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>target_or_use</t>
+          <t>catalog_number</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1730,19 +1730,19 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>What it targets or is used for (for example 'Western blot'); empty string if not stated.</t>
+          <t>Catalog number EXACTLY as printed; empty string if not reported. Never guess.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>corresponding_authors</t>
+          <t>reagents</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>target_or_use</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1753,7 +1753,7 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Author name as printed.</t>
+          <t>What it targets or is used for (for example 'Western blot'); empty string if not stated.</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>institution</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1776,34 +1776,30 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Institution given for this author; empty string if not stated. No email addresses.</t>
+          <t>Author name as printed.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>treatments</t>
+          <t>corresponding_authors</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>treatment</t>
+          <t>institution</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>pick-list</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Small-molecule drug; Biologic/antibody; Enzyme replacement; Gene therapy; Cell or stem-cell transplant; Surgery/procedure; Supportive care; Other</t>
-        </is>
-      </c>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>The treatment class.</t>
+          <t>Institution given for this author; empty string if not stated. No email addresses.</t>
         </is>
       </c>
     </row>
@@ -1815,30 +1811,34 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>treatment</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr"/>
+          <t>pick-list</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Small-molecule drug; Biologic/antibody; Enzyme replacement; Gene therapy; Cell or stem-cell transplant; Surgery/procedure; Supportive care; Other</t>
+        </is>
+      </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Specific drug or regimen (for example 'etanercept'); required if 'Other'; empty string if none.</t>
+          <t>The treatment class of ONE drug or regimen (one entry per drug).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>clinical_features</t>
+          <t>treatments</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>feature</t>
+          <t>detail</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1849,7 +1849,7 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>The clinical feature, as the paper words it.</t>
+          <t>The ONE specific drug or regimen (for example 'adalimumab'); required if 'Other'. Never list several drugs in one entry: add a separate entry for each drug.</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>detail</t>
+          <t>feature</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -1871,6 +1871,29 @@
       </c>
       <c r="D22" s="2" t="inlineStr"/>
       <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>The clinical feature, as the paper words it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>clinical_features</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>Optional extra detail (for example severity or age at onset); empty string if none.</t>
         </is>
@@ -1974,7 +1997,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Every entry needs evidence: a quote copied EXACTLY, character for character, from the paper text (at most about 300 characters; the single most informative phrase), the heading of the section it is in, and the page number from that section's marker (0 if unknown). Never paraphrase, never fix typos, never join text from different places.</t>
+          <t>Every entry needs evidence: a quote copied EXACTLY, character for character, from the paper text (at most about 300 characters; the single most informative phrase), the heading of the section it is in, and the page number from that section's marker (0 if unknown). Never paraphrase, never fix typos, never join text from different places. Choose the quote that shows what this paper itself did, studied or found; do not use a general definition or textbook description of the topic as the evidence for what the paper is about.</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2069,6 +2092,8 @@
     <col width="60" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2097,6 +2122,16 @@
           <t>Also send every section that starts on this page or earlier (0 = none)</t>
         </is>
       </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Re-read the whole paper when a category is not found? (Always / Only if key sections are missing / Never)</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Key sections (a re-read is skipped when the paper has any of these)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -2120,6 +2155,12 @@
       <c r="E2" s="2" t="n">
         <v>1</v>
       </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Always</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -2143,6 +2184,16 @@
       <c r="E3" s="2" t="n">
         <v>0</v>
       </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Only if key sections are missing</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>methods</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -2165,6 +2216,16 @@
       </c>
       <c r="E4" s="2" t="n">
         <v>0</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Only if key sections are missing</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>results; case</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>